<commit_message>
modifications to the forecasting query to bring token count down
</commit_message>
<xml_diff>
--- a/db/stockalerts.xlsx
+++ b/db/stockalerts.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,11 +451,11 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -466,11 +466,11 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -481,11 +481,11 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -496,11 +496,11 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>GD</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -511,11 +511,11 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -526,11 +526,11 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -541,11 +541,11 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -556,11 +556,11 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>V</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -571,11 +571,11 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46092</v>
+        <v>46094</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -586,11 +586,11 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46092</v>
+        <v>46094</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -601,11 +601,11 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -616,11 +616,11 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -631,11 +631,11 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,11 +646,11 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -661,11 +661,11 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -676,11 +676,11 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -691,11 +691,11 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -706,164 +706,14 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>NU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>AMZN</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>CAT</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>IBM</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>JNJ</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>MRK</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>3-Day Decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>NU</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
         <is>
           <t>3-Day Decline</t>
         </is>

</xml_diff>